<commit_message>
Dashboard 2026-09-07 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/32616334104/spec-32616334104.xlsx
+++ b/vse-loti/32616334104/spec-32616334104.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00&quot; ₽&quot;"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -58,12 +60,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -450,51 +455,94 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Наименование позиции (⌀ + s, если указано)</t>
+          <t>Наименование позиции</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>D×s, мм</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Кол-во (исх.)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ед. изм.</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Масса, т (приведённая)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Стоимость (без НДС)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Цена за т (без НДС)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Цена за т (с НДС)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Комплект технической документации (USB) 1 шт. Комплект инструментов для обслуживания 1 шт. Опорные площадки, комплект 1 шт. Осевой приводной блок 1 шт. Радиальный приводной блок 1 шт. Держатель расточного инструмента Ø40 3 шт. Резцедержатели для наружной обработки 25*25 1 шт. Оснащение: Резец DVJNR2525-M16, кол-во</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="3" t="n">
+        <v>90929492</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
+      <c r="G3" s="5" t="n">
+        <v>90929492</v>
+      </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Источник: Документация.docx</t>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>НМЦК из обоснования:</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>90929492</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Источник: spec-32616334104.txt</t>
         </is>
       </c>
     </row>

</xml_diff>